<commit_message>
Switch food menu to meal types
</commit_message>
<xml_diff>
--- a/templates/food-menu-event-tabs-template.xlsx
+++ b/templates/food-menu-event-tabs-template.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Haldi" sheetId="1" r:id="R547e2d1495d34e2d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sangeet" sheetId="2" r:id="R2a5d85b796e94e1a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pellikuthuru" sheetId="3" r:id="Rde0063b5881a4eba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Marriage" sheetId="4" r:id="Recc99c0588014b85"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Satyanarayana Swamy Vratam" sheetId="5" r:id="Rd9dfcb60c06c4cd0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Haldi" sheetId="1" r:id="R6841da9b23a545ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sangeet" sheetId="2" r:id="Ra09e1485468e4941"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pellikuthuru" sheetId="3" r:id="R5dfe8bd2ce464b12"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Marriage" sheetId="4" r:id="R956ee25fe28748cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Satyanarayana Swamy Vratam" sheetId="5" r:id="R2b73349e9fda4f75"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -262,7 +262,7 @@
   <x:autoFilter ref="A1:H101"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Dish"/>
-    <x:tableColumn id="2" name="Course Type"/>
+    <x:tableColumn id="2" name="Meal Type"/>
     <x:tableColumn id="3" name="Veg / Non-Veg"/>
     <x:tableColumn id="4" name="Cuisine"/>
     <x:tableColumn id="5" name="Cost"/>
@@ -279,7 +279,7 @@
   <x:autoFilter ref="A1:H101"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Dish"/>
-    <x:tableColumn id="2" name="Course Type"/>
+    <x:tableColumn id="2" name="Meal Type"/>
     <x:tableColumn id="3" name="Veg / Non-Veg"/>
     <x:tableColumn id="4" name="Cuisine"/>
     <x:tableColumn id="5" name="Cost"/>
@@ -296,7 +296,7 @@
   <x:autoFilter ref="A1:H101"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Dish"/>
-    <x:tableColumn id="2" name="Course Type"/>
+    <x:tableColumn id="2" name="Meal Type"/>
     <x:tableColumn id="3" name="Veg / Non-Veg"/>
     <x:tableColumn id="4" name="Cuisine"/>
     <x:tableColumn id="5" name="Cost"/>
@@ -313,7 +313,7 @@
   <x:autoFilter ref="A1:H101"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Dish"/>
-    <x:tableColumn id="2" name="Course Type"/>
+    <x:tableColumn id="2" name="Meal Type"/>
     <x:tableColumn id="3" name="Veg / Non-Veg"/>
     <x:tableColumn id="4" name="Cuisine"/>
     <x:tableColumn id="5" name="Cost"/>
@@ -330,7 +330,7 @@
   <x:autoFilter ref="A1:H101"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Dish"/>
-    <x:tableColumn id="2" name="Course Type"/>
+    <x:tableColumn id="2" name="Meal Type"/>
     <x:tableColumn id="3" name="Veg / Non-Veg"/>
     <x:tableColumn id="4" name="Cuisine"/>
     <x:tableColumn id="5" name="Cost"/>
@@ -552,7 +552,7 @@
         <x:v>Dish</x:v>
       </x:c>
       <x:c r="B1" s="6" t="str">
-        <x:v>Course Type</x:v>
+        <x:v>Meal Type</x:v>
       </x:c>
       <x:c r="C1" s="6" t="str">
         <x:v>Veg / Non-Veg</x:v>
@@ -1576,7 +1576,7 @@
   </x:sheetData>
   <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="B2:B101">
-      <x:formula1>"appetizers,snacks,mains,sides,desserts,beverages"</x:formula1>
+      <x:formula1>"breakfast,lunch,dinner"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="C2:C101">
       <x:formula1>"veg,non-veg,both"</x:formula1>
@@ -1587,7 +1587,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf5493b80505e47d4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R27b06342d4dd49ef"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1611,7 +1611,7 @@
         <x:v>Dish</x:v>
       </x:c>
       <x:c r="B1" s="6" t="str">
-        <x:v>Course Type</x:v>
+        <x:v>Meal Type</x:v>
       </x:c>
       <x:c r="C1" s="6" t="str">
         <x:v>Veg / Non-Veg</x:v>
@@ -2635,7 +2635,7 @@
   </x:sheetData>
   <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="B2:B101">
-      <x:formula1>"appetizers,snacks,mains,sides,desserts,beverages"</x:formula1>
+      <x:formula1>"breakfast,lunch,dinner"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="C2:C101">
       <x:formula1>"veg,non-veg,both"</x:formula1>
@@ -2646,7 +2646,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd8723a46e85142ba"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra95b7b6581184b41"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2670,7 +2670,7 @@
         <x:v>Dish</x:v>
       </x:c>
       <x:c r="B1" s="6" t="str">
-        <x:v>Course Type</x:v>
+        <x:v>Meal Type</x:v>
       </x:c>
       <x:c r="C1" s="6" t="str">
         <x:v>Veg / Non-Veg</x:v>
@@ -3694,7 +3694,7 @@
   </x:sheetData>
   <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="B2:B101">
-      <x:formula1>"appetizers,snacks,mains,sides,desserts,beverages"</x:formula1>
+      <x:formula1>"breakfast,lunch,dinner"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="C2:C101">
       <x:formula1>"veg,non-veg,both"</x:formula1>
@@ -3705,7 +3705,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re9023baa6efd4af4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6dd79fea03734afd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3729,7 +3729,7 @@
         <x:v>Dish</x:v>
       </x:c>
       <x:c r="B1" s="6" t="str">
-        <x:v>Course Type</x:v>
+        <x:v>Meal Type</x:v>
       </x:c>
       <x:c r="C1" s="6" t="str">
         <x:v>Veg / Non-Veg</x:v>
@@ -4753,7 +4753,7 @@
   </x:sheetData>
   <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="B2:B101">
-      <x:formula1>"appetizers,snacks,mains,sides,desserts,beverages"</x:formula1>
+      <x:formula1>"breakfast,lunch,dinner"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="C2:C101">
       <x:formula1>"veg,non-veg,both"</x:formula1>
@@ -4764,7 +4764,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58ba728f50e54458"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R471bb21571104938"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4788,7 +4788,7 @@
         <x:v>Dish</x:v>
       </x:c>
       <x:c r="B1" s="6" t="str">
-        <x:v>Course Type</x:v>
+        <x:v>Meal Type</x:v>
       </x:c>
       <x:c r="C1" s="6" t="str">
         <x:v>Veg / Non-Veg</x:v>
@@ -5812,7 +5812,7 @@
   </x:sheetData>
   <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="B2:B101">
-      <x:formula1>"appetizers,snacks,mains,sides,desserts,beverages"</x:formula1>
+      <x:formula1>"breakfast,lunch,dinner"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="C2:C101">
       <x:formula1>"veg,non-veg,both"</x:formula1>
@@ -5823,7 +5823,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R053ce6fc58984405"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf6ba0f0f91f54b7f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>